<commit_message>
Checkpoint: SeriesA cap table complete
</commit_message>
<xml_diff>
--- a/runs/20260415-113518/models/model.xlsx
+++ b/runs/20260415-113518/models/model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FED45268-A03D-6147-8652-3F294AE3BF43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{59718D00-AF7A-8A41-A87D-3EC8D926A087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="162" r:id="rId1"/>
     <sheet name="Detailed Cap Table" sheetId="163" r:id="rId2"/>
     <sheet name="SAFE Investments" sheetId="164" r:id="rId3"/>
+    <sheet name="SeriesA" sheetId="166" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="84">
   <si>
     <t>Total</t>
   </si>
@@ -193,17 +194,115 @@
     <t>Mark Lotke</t>
   </si>
   <si>
+    <t xml:space="preserve">Common </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option </t>
+  </si>
+  <si>
+    <t>Series A</t>
+  </si>
+  <si>
+    <t>Total Capitalization</t>
+  </si>
+  <si>
+    <t># of</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>Pool +</t>
+  </si>
+  <si>
+    <t>Total FD</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Invested</t>
+  </si>
+  <si>
+    <t>Pre A</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Common Stock and Options:</t>
+  </si>
+  <si>
+    <t>Total Common</t>
+  </si>
+  <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A Assumptions:</t>
+  </si>
+  <si>
+    <t>Total Raised</t>
+  </si>
+  <si>
+    <t>ESOP Issued &amp; Outstanding</t>
+  </si>
+  <si>
+    <t>ESOP Available</t>
+  </si>
+  <si>
+    <t>Other Series A</t>
+  </si>
+  <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price per Share </t>
+  </si>
+  <si>
+    <t>Other Common</t>
+  </si>
+  <si>
+    <t>SAFE Valuation Cap</t>
+  </si>
+  <si>
+    <t>Ten Eleven Ventures</t>
+  </si>
+  <si>
+    <t>SIDEKICK (THINK MORE SECURITY) &amp; TEN ELEVEN SERIES A</t>
+  </si>
+  <si>
+    <t>Other Investors</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="6">
+    <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0_-;_-[$$-409]* \(#,##0\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
+    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.0000_-;_-[$$-409]* \(#,##0.0000\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -339,6 +438,24 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -349,6 +466,19 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
       <family val="1"/>
     </font>
     <font>
@@ -377,8 +507,21 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFC0504D"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -558,8 +701,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -674,6 +823,156 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -719,50 +1018,176 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="19" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="175" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="5" fontId="19" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="175" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="37" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="29" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="29" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="29" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="29" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="24" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="19" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="19" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="24" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1181,610 +1606,610 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" s="5"/>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
+      <c r="A1" s="11"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="9" t="s">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="4"/>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="10"/>
+      <c r="B3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="10"/>
+      <c r="B4" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="25">
         <v>3600000</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="10">
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="25">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="26">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="6"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
-      <c r="B5" s="8" t="s">
+      <c r="A5" s="10"/>
+      <c r="B5" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="25">
         <v>3600000</v>
       </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="10">
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="25">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="26">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="6"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="10"/>
+      <c r="B6" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="25">
         <v>222187</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="10">
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="25">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="26">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="6"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="4"/>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="10"/>
+      <c r="B7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="25">
         <v>592500</v>
       </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="10">
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="25">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="26">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="6"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
-      <c r="B8" s="8" t="s">
+      <c r="A8" s="10"/>
+      <c r="B8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="25">
         <v>592500</v>
       </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="10">
+      <c r="D8" s="47"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="25">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="26">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="6"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="4"/>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="10"/>
+      <c r="B9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="25">
         <v>13500</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="47">
         <v>98900</v>
       </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="10">
+      <c r="E9" s="47"/>
+      <c r="F9" s="47"/>
+      <c r="G9" s="25">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="26">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="6"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="10"/>
+      <c r="B10" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="25">
         <v>9000</v>
       </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="10">
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="25">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="26">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="6"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
-      <c r="B11" s="8" t="s">
+      <c r="A11" s="10"/>
+      <c r="B11" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="14">
+      <c r="C11" s="25"/>
+      <c r="D11" s="47">
         <v>95000</v>
       </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="10">
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="25">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="26">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="6"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="8" t="s">
+      <c r="A12" s="10"/>
+      <c r="B12" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14">
+      <c r="C12" s="25"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47">
         <v>25000</v>
       </c>
-      <c r="F12" s="14"/>
-      <c r="G12" s="10">
+      <c r="F12" s="47"/>
+      <c r="G12" s="25">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12" s="26">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="6"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="4"/>
-      <c r="B13" s="8" t="s">
+      <c r="A13" s="10"/>
+      <c r="B13" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14">
+      <c r="C13" s="25"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="47">
         <v>41562</v>
       </c>
-      <c r="F13" s="14"/>
-      <c r="G13" s="10">
+      <c r="F13" s="47"/>
+      <c r="G13" s="25">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="26">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="6"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="8" t="s">
+      <c r="A14" s="10"/>
+      <c r="B14" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="14">
+      <c r="C14" s="25"/>
+      <c r="D14" s="47">
         <v>285000</v>
       </c>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="10">
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="25">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="26">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="6"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
-      <c r="B15" s="8" t="s">
+      <c r="A15" s="10"/>
+      <c r="B15" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="14">
+      <c r="C15" s="25"/>
+      <c r="D15" s="47">
         <v>50000</v>
       </c>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="10">
+      <c r="E15" s="47"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="25">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="26">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="6"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
-      <c r="B16" s="8" t="s">
+      <c r="A16" s="10"/>
+      <c r="B16" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="14">
+      <c r="C16" s="25"/>
+      <c r="D16" s="47">
         <v>285000</v>
       </c>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="10">
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
+      <c r="G16" s="25">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="26">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="6"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17" s="8" t="s">
+      <c r="A17" s="10"/>
+      <c r="B17" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14">
+      <c r="C17" s="25"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47">
         <v>96186</v>
       </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="10">
+      <c r="F17" s="47"/>
+      <c r="G17" s="25">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="11">
+      <c r="H17" s="26">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="6"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="4"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="8" t="s">
+      <c r="A18" s="10"/>
+      <c r="B18" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14">
+      <c r="C18" s="25"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47">
         <v>48095</v>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="10">
+      <c r="F18" s="47"/>
+      <c r="G18" s="25">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="11">
+      <c r="H18" s="26">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="6"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
-      <c r="B19" s="8" t="s">
+      <c r="A19" s="10"/>
+      <c r="B19" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14">
+      <c r="C19" s="25"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47">
         <v>12395</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="25">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="11">
+      <c r="H19" s="26">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="6"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="B20" s="8" t="s">
+      <c r="A20" s="10"/>
+      <c r="B20" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14">
+      <c r="C20" s="25"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="47">
         <v>8333</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="25">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="11">
+      <c r="H20" s="26">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="6"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="4"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
     </row>
     <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
-      <c r="B21" s="8" t="s">
+      <c r="A21" s="10"/>
+      <c r="B21" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="14">
+      <c r="C21" s="25"/>
+      <c r="D21" s="47">
         <v>65105</v>
       </c>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="10">
+      <c r="E21" s="47"/>
+      <c r="F21" s="47"/>
+      <c r="G21" s="25">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="11">
+      <c r="H21" s="26">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="6"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="4"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
     </row>
     <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
-      <c r="B23" s="16" t="s">
+      <c r="A23" s="10"/>
+      <c r="B23" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="53">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="53">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="53">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="53">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="15">
+      <c r="G23" s="53">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="6"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1804,402 +2229,1081 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="2"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+      <c r="A1" s="5"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="2"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="7" t="s">
+      <c r="A2" s="5"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="2"/>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="9" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="2"/>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="28">
         <v>25000</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="8" t="s">
+      <c r="D4" s="5"/>
+      <c r="E4" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="2"/>
-      <c r="B5" s="8" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="28">
         <v>25000</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="2"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="28">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="28">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="5"/>
+      <c r="B8" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="28">
+        <v>16566</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="5"/>
+      <c r="B9" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="28">
+        <v>250000</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="5"/>
+      <c r="B10" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="28">
+        <v>100000</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="5"/>
+      <c r="B11" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="28">
+        <v>300000</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="5"/>
+      <c r="B12" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="28">
+        <v>37500</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="5"/>
+      <c r="B13" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="28">
+        <v>250000</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="5"/>
+      <c r="B14" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="28">
+        <v>100000</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="5"/>
+      <c r="B15" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="28">
+        <v>41164</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="28">
+        <v>2328778</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="5"/>
+      <c r="B17" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="28">
+        <v>1506000</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
+      <c r="B18" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="28">
+        <v>50000</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+    </row>
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="5"/>
+      <c r="B19" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="28">
+        <v>212500</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="5"/>
+      <c r="B20" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="28">
+        <v>25000</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="5"/>
+      <c r="B21" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="28">
+        <v>61746</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
+      <c r="B22" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="28">
+        <v>100000</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="5"/>
+      <c r="B23" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="28">
+        <v>100000</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
+      <c r="B24" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="28">
+        <v>61746</v>
+      </c>
+      <c r="D24" s="5"/>
+      <c r="E24" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="5"/>
+      <c r="B25" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="28">
+        <v>250000</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="5"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="5"/>
+      <c r="B27" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="27">
+        <f>SUM(C4:C25)</f>
+        <v>9825000</v>
+      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{886C911D-37FD-D94E-8729-EB65E9AACF33}">
+  <dimension ref="A1:N33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="3.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.5" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="3.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="3.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" customWidth="1"/>
+    <col min="13" max="13" width="9.33203125" customWidth="1"/>
+    <col min="14" max="14" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="62"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="61"/>
+      <c r="L2" s="61"/>
+      <c r="M2" s="61"/>
+      <c r="N2" s="62"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A3" s="1"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="61"/>
+      <c r="M3" s="61"/>
+      <c r="N3" s="62"/>
+    </row>
+    <row r="4" spans="1:14" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+      <c r="B4" s="61" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="61"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="61"/>
+      <c r="M4" s="61"/>
+      <c r="N4" s="62"/>
+    </row>
+    <row r="5" spans="1:14" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="63" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="63"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="63"/>
+      <c r="L5" s="63"/>
+      <c r="M5" s="63"/>
+      <c r="N5" s="62"/>
+    </row>
+    <row r="6" spans="1:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="58"/>
+      <c r="C6" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="68"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" s="68"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="K6" s="73"/>
+      <c r="L6" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="M6" s="55"/>
+      <c r="N6" s="30"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="66" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="30"/>
+      <c r="G7" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="42" t="s">
+        <v>58</v>
+      </c>
       <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="2"/>
-      <c r="B8" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="13">
-        <v>16566</v>
-      </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
+      <c r="J7" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="K7" s="41"/>
+      <c r="L7" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="M7" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="N7" s="30"/>
+    </row>
+    <row r="8" spans="1:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="64"/>
+      <c r="C8" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" s="30"/>
+      <c r="G8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H8" s="40" t="s">
+        <v>62</v>
+      </c>
       <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="13">
-        <v>250000</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="2"/>
-      <c r="B10" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="13">
-        <v>100000</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="1"/>
+      <c r="J8" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="K8" s="43"/>
+      <c r="L8" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="M8" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="N8" s="30"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="65" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="54"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="1"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="44" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="8">
+        <f>'Detailed Cap Table'!C4</f>
+        <v>3600000</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
       <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
+      <c r="J10" s="3"/>
       <c r="K10" s="1"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="2"/>
-      <c r="B11" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="13">
-        <v>300000</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="8" t="s">
-        <v>28</v>
-      </c>
+      <c r="L10" s="31">
+        <f>C10+E10+H10+J10</f>
+        <v>3600000</v>
+      </c>
+      <c r="M10" s="51">
+        <f ca="1">L10/$L$22</f>
+        <v>0.19407509228944511</v>
+      </c>
+      <c r="N10" s="1"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="44" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="8">
+        <f>'Detailed Cap Table'!C5</f>
+        <v>3600000</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="J11" s="3"/>
       <c r="K11" s="1"/>
-    </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="2"/>
-      <c r="B12" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="13">
-        <v>37500</v>
-      </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="8" t="s">
-        <v>36</v>
-      </c>
+      <c r="L11" s="31">
+        <f>C11+E11+H11+J11</f>
+        <v>3600000</v>
+      </c>
+      <c r="M11" s="51">
+        <f ca="1">L11/$L$22</f>
+        <v>0.19407509228944511</v>
+      </c>
+      <c r="N11" s="1"/>
+    </row>
+    <row r="12" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="8">
+        <f>'Detailed Cap Table'!C23-'Detailed Cap Table'!C4-'Detailed Cap Table'!C5+'Detailed Cap Table'!D23-'Detailed Cap Table'!D21+'Detailed Cap Table'!F23</f>
+        <v>2264315</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
+      <c r="J12" s="3"/>
       <c r="K12" s="1"/>
-    </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="13">
-        <v>250000</v>
-      </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="1"/>
+      <c r="L12" s="31">
+        <f>C12+E12+H12+J12</f>
+        <v>2264315</v>
+      </c>
+      <c r="M12" s="51">
+        <f ca="1">L12/$L$22</f>
+        <v>0.12206865072149302</v>
+      </c>
+      <c r="N12" s="1"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="8">
+        <f>'Detailed Cap Table'!E23</f>
+        <v>210843</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
+      <c r="J13" s="3"/>
       <c r="K13" s="1"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="2"/>
-      <c r="B14" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="13">
-        <v>100000</v>
-      </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="1"/>
+      <c r="L13" s="31">
+        <f>C13+E13+H13+J13</f>
+        <v>210843</v>
+      </c>
+      <c r="M13" s="51">
+        <f ca="1">L13/$L$22</f>
+        <v>1.1366492967662076E-2</v>
+      </c>
+      <c r="N13" s="1"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="44" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="8">
+        <f>'Detailed Cap Table'!D21</f>
+        <v>65105</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
+      <c r="J14" s="31">
+        <f ca="1">IFERROR(ROUND(0.1*L22-C14,0),0)</f>
+        <v>1789847</v>
+      </c>
       <c r="K14" s="1"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="13">
-        <v>41164</v>
-      </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="8" t="s">
-        <v>52</v>
+      <c r="L14" s="31">
+        <f ca="1">C14+E14+H14+J14</f>
+        <v>1854952</v>
+      </c>
+      <c r="M14" s="51">
+        <f ca="1">L14/$L$22</f>
+        <v>9.9999994609025214E-2</v>
+      </c>
+      <c r="N14" s="1"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="69">
+        <f>SUM(C10:C14)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D15" s="3">
+        <f>SUM(D10:D14)</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="3">
+        <f>SUM(E10:E14)</f>
+        <v>0</v>
       </c>
       <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
+      <c r="G15" s="3">
+        <f>SUM(G10:G14)</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="3">
+        <f>SUM(H10:H14)</f>
+        <v>0</v>
+      </c>
       <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
+      <c r="J15" s="3">
+        <f ca="1">SUM(J10:J14)</f>
+        <v>1789847</v>
+      </c>
       <c r="K15" s="1"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="2"/>
-      <c r="B16" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="13">
-        <v>2328778</v>
-      </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="8" t="s">
-        <v>52</v>
-      </c>
+      <c r="L15" s="31">
+        <f ca="1">SUM(L10:L14)</f>
+        <v>11530110</v>
+      </c>
+      <c r="M15" s="49">
+        <f ca="1">L15/$L$22</f>
+        <v>0.62158532287707047</v>
+      </c>
+      <c r="N15" s="1"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="45" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
       <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
+      <c r="J16" s="3"/>
       <c r="K16" s="1"/>
-    </row>
-    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="13">
-        <v>1506000</v>
-      </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="8" t="s">
+      <c r="L16" s="3"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="1"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="44" t="s">
         <v>42</v>
       </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="32">
+        <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C17+'SAFE Investments'!C16+'SAFE Investments'!C15+'SAFE Investments'!C21+'SAFE Investments'!C24+'SAFE Investments'!C8</f>
+        <v>8000000</v>
+      </c>
+      <c r="E17" s="31">
+        <f>IFERROR(ROUND(D17/$E$24,0),0)</f>
+        <v>1939567</v>
+      </c>
       <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
+      <c r="G17" s="74">
+        <v>5000000</v>
+      </c>
+      <c r="H17" s="31">
+        <f ca="1">IFERROR(ROUND(G17/$H$24,0),0)</f>
+        <v>1159345</v>
+      </c>
       <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
+      <c r="J17" s="3"/>
       <c r="K17" s="1"/>
-    </row>
-    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="2"/>
-      <c r="B18" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="13">
-        <v>50000</v>
-      </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="1"/>
+      <c r="L17" s="31">
+        <f ca="1">C17+E17+H17+J17</f>
+        <v>3098912</v>
+      </c>
+      <c r="M17" s="51">
+        <f ca="1">L17/$L$22</f>
+        <v>0.16706156455468579</v>
+      </c>
+      <c r="N17" s="1"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="44" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="32">
+        <f>'SAFE Investments'!C27-D17</f>
+        <v>1825000</v>
+      </c>
+      <c r="E18" s="31">
+        <f>IFERROR(ROUND(D18/$E$24,0),0)</f>
+        <v>442464</v>
+      </c>
       <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="31"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
+      <c r="J18" s="3"/>
       <c r="K18" s="1"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="13">
-        <v>212500</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="8" t="s">
-        <v>36</v>
-      </c>
+      <c r="L18" s="31">
+        <f>C18+E18+H18+J18</f>
+        <v>442464</v>
+      </c>
+      <c r="M18" s="51">
+        <f ca="1">L18/$L$22</f>
+        <v>2.3853122676321399E-2</v>
+      </c>
+      <c r="N18" s="1"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="44" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="7"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
       <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
+      <c r="G19" s="74">
+        <v>12000000</v>
+      </c>
+      <c r="H19" s="31">
+        <f ca="1">IFERROR(ROUND(G19/$H$24,0),0)</f>
+        <v>2782428</v>
+      </c>
       <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
+      <c r="J19" s="3"/>
       <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="2"/>
-      <c r="B20" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="13">
-        <v>25000</v>
-      </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="1"/>
+      <c r="L19" s="31">
+        <f ca="1">C19+E19+H19+J19</f>
+        <v>2782428</v>
+      </c>
+      <c r="M19" s="51">
+        <f ca="1">L19/$L$22</f>
+        <v>0.14999999191353783</v>
+      </c>
+      <c r="N19" s="1"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="44" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="7"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
       <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
+      <c r="G20" s="74">
+        <v>3000000</v>
+      </c>
+      <c r="H20" s="31">
+        <f ca="1">IFERROR(ROUND(G20/$H$24,0),0)</f>
+        <v>695607</v>
+      </c>
       <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
+      <c r="J20" s="3"/>
       <c r="K20" s="1"/>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="2"/>
-      <c r="B21" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="13">
-        <v>61746</v>
-      </c>
-      <c r="D21" s="2"/>
-      <c r="E21" s="8" t="s">
-        <v>52</v>
-      </c>
+      <c r="L20" s="31">
+        <f ca="1">C20+E20+H20+J20</f>
+        <v>695607</v>
+      </c>
+      <c r="M20" s="51">
+        <f ca="1">L20/$L$22</f>
+        <v>3.7499997978384457E-2</v>
+      </c>
+      <c r="N20" s="1"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A21" s="1"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
       <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
+      <c r="J21" s="3"/>
       <c r="K21" s="1"/>
-    </row>
-    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="2"/>
-      <c r="B22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="13">
-        <v>100000</v>
-      </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="1"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="1"/>
+    </row>
+    <row r="22" spans="1:14" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="45" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="16">
+        <f>C15+SUM(C17:C20)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D22" s="71">
+        <f>SUM(D10:D20)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E22" s="16">
+        <f>SUM(E10:E20)</f>
+        <v>2382031</v>
+      </c>
       <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
+      <c r="G22" s="72">
+        <f>SUM(G10:G20)</f>
+        <v>20000000</v>
+      </c>
+      <c r="H22" s="16">
+        <f ca="1">SUM(H10:H20)</f>
+        <v>4637380</v>
+      </c>
       <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
+      <c r="J22" s="15">
+        <f ca="1">J14</f>
+        <v>1789847</v>
+      </c>
       <c r="K22" s="1"/>
-    </row>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="2"/>
-      <c r="B23" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C23" s="13">
-        <v>100000</v>
-      </c>
-      <c r="D23" s="2"/>
+      <c r="L22" s="16">
+        <f ca="1">SUM(L17:L20)+L15</f>
+        <v>18549521</v>
+      </c>
+      <c r="M22" s="52">
+        <f ca="1">SUM(M17:M20)+M15</f>
+        <v>0.99999999999999989</v>
+      </c>
+      <c r="N22" s="1"/>
+    </row>
+    <row r="23" spans="1:14" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
@@ -2207,68 +3311,86 @@
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
-    </row>
-    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="2"/>
-      <c r="B24" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="13">
-        <v>61746</v>
-      </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="8" t="s">
-        <v>52</v>
+      <c r="L23" s="1"/>
+      <c r="M23" s="56"/>
+      <c r="N23" s="1"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A24" s="1"/>
+      <c r="B24" s="44" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="14">
+        <f>(C31-D22)/'Detailed Cap Table'!G23</f>
+        <v>4.1246319529565065</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
+      <c r="H24" s="60">
+        <f ca="1">IFERROR(H26/L22,0)</f>
+        <v>4.3127798286543353</v>
+      </c>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
-    </row>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="2"/>
-      <c r="B25" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="13">
-        <v>250000</v>
-      </c>
-      <c r="D25" s="2"/>
-      <c r="E25" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-      <c r="K25" s="1"/>
-    </row>
-    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="2"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="56"/>
+      <c r="N24" s="1"/>
+    </row>
+    <row r="25" spans="1:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="46" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="70">
+        <f>E26-D22</f>
+        <v>40175000</v>
+      </c>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="70">
+        <f>H26-G22</f>
+        <v>60000000</v>
+      </c>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="57"/>
+      <c r="N25" s="1"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A26" s="1"/>
+      <c r="B26" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="75">
+        <v>50000000</v>
+      </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
+      <c r="H26" s="76">
+        <f>C29+C30</f>
+        <v>80000000</v>
+      </c>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
-    </row>
-    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="2"/>
-      <c r="B27" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="C27" s="12">
-        <f>SUM(C4:C25)</f>
-        <v>9825000</v>
-      </c>
-      <c r="D27" s="2"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
@@ -2276,6 +3398,121 @@
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+      <c r="B29" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="48">
+        <v>60000000</v>
+      </c>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+      <c r="B30" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C30" s="48">
+        <v>20000000</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+      <c r="B31" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C31" s="48">
+        <v>50000000</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: SAFE Investments complete
</commit_message>
<xml_diff>
--- a/runs/20260415-113518/models/model.xlsx
+++ b/runs/20260415-113518/models/model.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F17A8F5D-DF94-C84E-85C4-23D90490A0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8257EF7-422C-684F-90F8-EF14BBE11B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet9" sheetId="168" r:id="rId1"/>
     <sheet name="Detailed Cap Table" sheetId="169" r:id="rId2"/>
+    <sheet name="SAFE Investments" sheetId="170" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
   <si>
     <t>Total</t>
   </si>
@@ -112,13 +113,97 @@
   </si>
   <si>
     <t>Available Options</t>
+  </si>
+  <si>
+    <t>SAFE</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>IRA is actual investor</t>
+  </si>
+  <si>
+    <t>Accomplice Founder Fund, L.P.</t>
+  </si>
+  <si>
+    <t>Accomplice Fund IV, L.P</t>
+  </si>
+  <si>
+    <t>Amir Bagherzadeh</t>
+  </si>
+  <si>
+    <t>Elizabeth A. Donaghey Irrevocable Trust 2016</t>
+  </si>
+  <si>
+    <t>Gunderson Partners</t>
+  </si>
+  <si>
+    <t>Joe Arcadi</t>
+  </si>
+  <si>
+    <t>Kamal Ravikant Capital, LP - E4</t>
+  </si>
+  <si>
+    <t>Navel</t>
+  </si>
+  <si>
+    <t>Maria Cirino</t>
+  </si>
+  <si>
+    <t>Mike Viscuso</t>
+  </si>
+  <si>
+    <t>Mozart Holdings, LLC</t>
+  </si>
+  <si>
+    <t>Orcinus Generational Irrevocable Trust - 2024</t>
+  </si>
+  <si>
+    <t>Owl Rock Capital III, LLC</t>
+  </si>
+  <si>
+    <t>Accomplice</t>
+  </si>
+  <si>
+    <t>Ralph Folz</t>
+  </si>
+  <si>
+    <t>Ravikant Capital, LP - F3</t>
+  </si>
+  <si>
+    <t>Sean Leach</t>
+  </si>
+  <si>
+    <t>The Francis V. Castellucci Trust - 2020</t>
+  </si>
+  <si>
+    <t>The Patrick M. Morley 1999 Trust,</t>
+  </si>
+  <si>
+    <t>Tom Barsi</t>
+  </si>
+  <si>
+    <t>Travis MacInnes</t>
+  </si>
+  <si>
+    <t>UWS West End Family Trust</t>
+  </si>
+  <si>
+    <t>Mark Lotke</t>
+  </si>
+  <si>
+    <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+  </numFmts>
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -252,6 +337,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -614,31 +712,47 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1058,9 +1172,517 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="5"/>
+      <c r="B4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10">
+        <v>3600000</v>
+      </c>
+      <c r="D4" s="14"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="10">
+        <f>SUM(C4:F4)</f>
+        <v>3600000</v>
+      </c>
+      <c r="H4" s="11">
+        <f>G4/$G$23</f>
+        <v>0.36959987630724139</v>
+      </c>
+      <c r="I4" s="6"/>
+      <c r="J4" s="5"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="5"/>
+      <c r="B5" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="10">
+        <v>3600000</v>
+      </c>
+      <c r="D5" s="14"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="10">
+        <f>SUM(C5:F5)</f>
+        <v>3600000</v>
+      </c>
+      <c r="H5" s="11">
+        <f>G5/$G$23</f>
+        <v>0.36959987630724139</v>
+      </c>
+      <c r="I5" s="6"/>
+      <c r="J5" s="5"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="5"/>
+      <c r="B6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="10">
+        <v>222187</v>
+      </c>
+      <c r="D6" s="14"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="10">
+        <f>SUM(C6:F6)</f>
+        <v>222187</v>
+      </c>
+      <c r="H6" s="11">
+        <f>G6/$G$23</f>
+        <v>2.28111910325214E-2</v>
+      </c>
+      <c r="I6" s="6"/>
+      <c r="J6" s="5"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="5"/>
+      <c r="B7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="10">
+        <v>592500</v>
+      </c>
+      <c r="D7" s="14"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="10">
+        <f>SUM(C7:F7)</f>
+        <v>592500</v>
+      </c>
+      <c r="H7" s="11">
+        <f>G7/$G$23</f>
+        <v>6.0829979642233481E-2</v>
+      </c>
+      <c r="I7" s="6"/>
+      <c r="J7" s="5"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" s="5"/>
+      <c r="B8" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="10">
+        <v>592500</v>
+      </c>
+      <c r="D8" s="14"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="10">
+        <f>SUM(C8:F8)</f>
+        <v>592500</v>
+      </c>
+      <c r="H8" s="11">
+        <f>G8/$G$23</f>
+        <v>6.0829979642233481E-2</v>
+      </c>
+      <c r="I8" s="6"/>
+      <c r="J8" s="5"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" s="5"/>
+      <c r="B9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="10">
+        <v>13500</v>
+      </c>
+      <c r="D9" s="10">
+        <v>98900</v>
+      </c>
+      <c r="E9" s="14"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="10">
+        <f>SUM(C9:F9)</f>
+        <v>112400</v>
+      </c>
+      <c r="H9" s="11">
+        <f>G9/$G$23</f>
+        <v>1.1539729471370537E-2</v>
+      </c>
+      <c r="I9" s="6"/>
+      <c r="J9" s="5"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="5"/>
+      <c r="B10" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="10">
+        <v>9000</v>
+      </c>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="10">
+        <f>SUM(C10:F10)</f>
+        <v>9000</v>
+      </c>
+      <c r="H10" s="11">
+        <f>G10/$G$23</f>
+        <v>9.2399969076810353E-4</v>
+      </c>
+      <c r="I10" s="6"/>
+      <c r="J10" s="5"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" s="5"/>
+      <c r="B11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="14"/>
+      <c r="D11" s="10">
+        <v>95000</v>
+      </c>
+      <c r="E11" s="14"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="10">
+        <f>SUM(C11:F11)</f>
+        <v>95000</v>
+      </c>
+      <c r="H11" s="11">
+        <f>G11/$G$23</f>
+        <v>9.7533300692188695E-3</v>
+      </c>
+      <c r="I11" s="6"/>
+      <c r="J11" s="5"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" s="5"/>
+      <c r="B12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="10">
+        <v>25000</v>
+      </c>
+      <c r="F12" s="14"/>
+      <c r="G12" s="10">
+        <f>SUM(C12:F12)</f>
+        <v>25000</v>
+      </c>
+      <c r="H12" s="11">
+        <f>G12/$G$23</f>
+        <v>2.5666658076891765E-3</v>
+      </c>
+      <c r="I12" s="6"/>
+      <c r="J12" s="5"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" s="5"/>
+      <c r="B13" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="10">
+        <v>41562</v>
+      </c>
+      <c r="F13" s="14"/>
+      <c r="G13" s="10">
+        <f>SUM(C13:F13)</f>
+        <v>41562</v>
+      </c>
+      <c r="H13" s="11">
+        <f>G13/$G$23</f>
+        <v>4.2670305719671019E-3</v>
+      </c>
+      <c r="I13" s="6"/>
+      <c r="J13" s="5"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" s="5"/>
+      <c r="B14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="14"/>
+      <c r="D14" s="10">
+        <v>285000</v>
+      </c>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="10">
+        <f>SUM(C14:F14)</f>
+        <v>285000</v>
+      </c>
+      <c r="H14" s="11">
+        <f>G14/$G$23</f>
+        <v>2.925999020765661E-2</v>
+      </c>
+      <c r="I14" s="6"/>
+      <c r="J14" s="5"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" s="5"/>
+      <c r="B15" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="14"/>
+      <c r="D15" s="10">
+        <v>50000</v>
+      </c>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="10">
+        <f>SUM(C15:F15)</f>
+        <v>50000</v>
+      </c>
+      <c r="H15" s="11">
+        <f>G15/$G$23</f>
+        <v>5.133331615378353E-3</v>
+      </c>
+      <c r="I15" s="6"/>
+      <c r="J15" s="5"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="14"/>
+      <c r="D16" s="10">
+        <v>285000</v>
+      </c>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="10">
+        <f>SUM(C16:F16)</f>
+        <v>285000</v>
+      </c>
+      <c r="H16" s="11">
+        <f>G16/$G$23</f>
+        <v>2.925999020765661E-2</v>
+      </c>
+      <c r="I16" s="6"/>
+      <c r="J16" s="5"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" s="5"/>
+      <c r="B17" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="10">
+        <v>96186</v>
+      </c>
+      <c r="F17" s="14"/>
+      <c r="G17" s="10">
+        <f>SUM(C17:F17)</f>
+        <v>96186</v>
+      </c>
+      <c r="H17" s="11">
+        <f>G17/$G$23</f>
+        <v>9.8750926951356455E-3</v>
+      </c>
+      <c r="I17" s="6"/>
+      <c r="J17" s="5"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
+      <c r="B18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="10">
+        <v>48095</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="10">
+        <f>SUM(C18:F18)</f>
+        <v>48095</v>
+      </c>
+      <c r="H18" s="11">
+        <f>G18/$G$23</f>
+        <v>4.9377516808324371E-3</v>
+      </c>
+      <c r="I18" s="6"/>
+      <c r="J18" s="5"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" s="5"/>
+      <c r="B19" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="10">
+        <v>12395</v>
+      </c>
+      <c r="G19" s="10">
+        <f>SUM(C19:F19)</f>
+        <v>12395</v>
+      </c>
+      <c r="H19" s="11">
+        <f>G19/$G$23</f>
+        <v>1.2725529074522936E-3</v>
+      </c>
+      <c r="I19" s="6"/>
+      <c r="J19" s="5"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" s="5"/>
+      <c r="B20" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="10">
+        <v>8333</v>
+      </c>
+      <c r="G20" s="10">
+        <f>SUM(C20:F20)</f>
+        <v>8333</v>
+      </c>
+      <c r="H20" s="11">
+        <f>G20/$G$23</f>
+        <v>8.5552104701895626E-4</v>
+      </c>
+      <c r="I20" s="6"/>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="5"/>
+      <c r="B21" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="14"/>
+      <c r="D21" s="10">
+        <v>65105</v>
+      </c>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="10">
+        <f>SUM(C21:F21)</f>
+        <v>65105</v>
+      </c>
+      <c r="H21" s="11">
+        <f>G21/$G$23</f>
+        <v>6.6841110963841528E-3</v>
+      </c>
+      <c r="I21" s="6"/>
+      <c r="J21" s="5"/>
+    </row>
+    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="5"/>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="5"/>
+      <c r="B23" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23" s="15">
+        <f>SUM(C4:C21)</f>
+        <v>8629687</v>
+      </c>
+      <c r="D23" s="15">
+        <f>SUM(D4:D21)</f>
+        <v>879005</v>
+      </c>
+      <c r="E23" s="15">
+        <f>SUM(E4:E21)</f>
+        <v>210843</v>
+      </c>
+      <c r="F23" s="15">
+        <f>SUM(F4:F21)</f>
+        <v>20728</v>
+      </c>
+      <c r="G23" s="15">
+        <f>SUM(G4:G21)</f>
+        <v>9740263</v>
+      </c>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C41D99B4-134A-FB41-B826-C99A5893907A}">
+  <dimension ref="A1:K27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="2" max="2" width="51.33203125" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="4" max="4" width="3.33203125" customWidth="1"/>
+    <col min="5" max="5" width="60.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="C1" s="3"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -1068,485 +1690,466 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="C2" s="7"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="5" t="s">
-        <v>1</v>
-      </c>
+      <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="C3" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K3" s="2"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
-      <c r="B4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="6">
-        <f>SUM(C4:F4)</f>
-        <v>3600000</v>
-      </c>
-      <c r="H4" s="7">
-        <f>G4/$G$23</f>
-        <v>0.36959987630724139</v>
-      </c>
-      <c r="I4" s="3"/>
+      <c r="B4" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="13">
+        <v>25000</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K4" s="2"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
-      <c r="B5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="6">
-        <f>SUM(C5:F5)</f>
-        <v>3600000</v>
-      </c>
-      <c r="H5" s="7">
-        <f>G5/$G$23</f>
-        <v>0.36959987630724139</v>
-      </c>
-      <c r="I5" s="3"/>
+      <c r="B5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="13">
+        <v>25000</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K5" s="2"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
-      <c r="B6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="6">
-        <v>222187</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="6">
-        <f>SUM(C6:F6)</f>
-        <v>222187</v>
-      </c>
-      <c r="H6" s="7">
-        <f>G6/$G$23</f>
-        <v>2.28111910325214E-2</v>
-      </c>
-      <c r="I6" s="3"/>
+      <c r="B6" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="13">
+        <v>137170.75</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K6" s="2"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
-      <c r="B7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="6">
-        <v>592500</v>
-      </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="6">
-        <f>SUM(C7:F7)</f>
-        <v>592500</v>
-      </c>
-      <c r="H7" s="7">
-        <f>G7/$G$23</f>
-        <v>6.0829979642233481E-2</v>
-      </c>
-      <c r="I7" s="3"/>
+      <c r="B7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="13">
+        <v>3846829.25</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K7" s="2"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="6">
-        <v>592500</v>
-      </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="6">
-        <f>SUM(C8:F8)</f>
-        <v>592500</v>
-      </c>
-      <c r="H8" s="7">
-        <f>G8/$G$23</f>
-        <v>6.0829979642233481E-2</v>
-      </c>
-      <c r="I8" s="3"/>
+      <c r="B8" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="13">
+        <v>16566</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K8" s="2"/>
+    </row>
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
-      <c r="B9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="6">
-        <v>13500</v>
-      </c>
-      <c r="D9" s="6">
-        <v>98900</v>
-      </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="6">
-        <f>SUM(C9:F9)</f>
-        <v>112400</v>
-      </c>
-      <c r="H9" s="7">
-        <f>G9/$G$23</f>
-        <v>1.1539729471370537E-2</v>
-      </c>
-      <c r="I9" s="3"/>
+      <c r="B9" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="13">
+        <v>250000</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K9" s="2"/>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
-      <c r="B10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="6">
-        <v>9000</v>
-      </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="6">
-        <f>SUM(C10:F10)</f>
-        <v>9000</v>
-      </c>
-      <c r="H10" s="7">
-        <f>G10/$G$23</f>
-        <v>9.2399969076810353E-4</v>
-      </c>
-      <c r="I10" s="3"/>
+      <c r="B10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="13">
+        <v>100000</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K10" s="2"/>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
-      <c r="B11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="6">
-        <v>95000</v>
-      </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="6">
-        <f>SUM(C11:F11)</f>
-        <v>95000</v>
-      </c>
-      <c r="H11" s="7">
-        <f>G11/$G$23</f>
-        <v>9.7533300692188695E-3</v>
-      </c>
-      <c r="I11" s="3"/>
+      <c r="B11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="13">
+        <v>300000</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K11" s="2"/>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
-      <c r="B12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="6">
+      <c r="B12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="13">
+        <v>37500</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="13">
+        <v>250000</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="2"/>
+      <c r="B14" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="13">
+        <v>100000</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="2"/>
+      <c r="B15" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="13">
+        <v>41164</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="2"/>
+      <c r="B16" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="13">
+        <v>2328778</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="2"/>
+      <c r="B17" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="13">
+        <v>1506000</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="2"/>
+      <c r="B18" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="13">
+        <v>50000</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+    </row>
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="2"/>
+      <c r="B19" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="13">
+        <v>212500</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="2"/>
+      <c r="B20" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="13">
         <v>25000</v>
       </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="6">
-        <f>SUM(C12:F12)</f>
-        <v>25000</v>
-      </c>
-      <c r="H12" s="7">
-        <f>G12/$G$23</f>
-        <v>2.5666658076891765E-3</v>
-      </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="6">
-        <v>41562</v>
-      </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="6">
-        <f>SUM(C13:F13)</f>
-        <v>41562</v>
-      </c>
-      <c r="H13" s="7">
-        <f>G13/$G$23</f>
-        <v>4.2670305719671019E-3</v>
-      </c>
-      <c r="I13" s="3"/>
-      <c r="J13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="2"/>
-      <c r="B14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="6">
-        <v>285000</v>
-      </c>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="6">
-        <f>SUM(C14:F14)</f>
-        <v>285000</v>
-      </c>
-      <c r="H14" s="7">
-        <f>G14/$G$23</f>
-        <v>2.925999020765661E-2</v>
-      </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="6">
-        <v>50000</v>
-      </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="6">
-        <f>SUM(C15:F15)</f>
-        <v>50000</v>
-      </c>
-      <c r="H15" s="7">
-        <f>G15/$G$23</f>
-        <v>5.133331615378353E-3</v>
-      </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="2"/>
-      <c r="B16" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="6">
-        <v>285000</v>
-      </c>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="6">
-        <f>SUM(C16:F16)</f>
-        <v>285000</v>
-      </c>
-      <c r="H16" s="7">
-        <f>G16/$G$23</f>
-        <v>2.925999020765661E-2</v>
-      </c>
-      <c r="I16" s="3"/>
-      <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="6">
-        <v>96186</v>
-      </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="6">
-        <f>SUM(C17:F17)</f>
-        <v>96186</v>
-      </c>
-      <c r="H17" s="7">
-        <f>G17/$G$23</f>
-        <v>9.8750926951356455E-3</v>
-      </c>
-      <c r="I17" s="3"/>
-      <c r="J17" s="2"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="2"/>
-      <c r="B18" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="6">
-        <v>48095</v>
-      </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="6">
-        <f>SUM(C18:F18)</f>
-        <v>48095</v>
-      </c>
-      <c r="H18" s="7">
-        <f>G18/$G$23</f>
-        <v>4.9377516808324371E-3</v>
-      </c>
-      <c r="I18" s="3"/>
-      <c r="J18" s="2"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="6">
-        <v>12395</v>
-      </c>
-      <c r="G19" s="6">
-        <f>SUM(C19:F19)</f>
-        <v>12395</v>
-      </c>
-      <c r="H19" s="7">
-        <f>G19/$G$23</f>
-        <v>1.2725529074522936E-3</v>
-      </c>
-      <c r="I19" s="3"/>
-      <c r="J19" s="2"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="2"/>
-      <c r="B20" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="6">
-        <v>8333</v>
-      </c>
-      <c r="G20" s="6">
-        <f>SUM(C20:F20)</f>
-        <v>8333</v>
-      </c>
-      <c r="H20" s="7">
-        <f>G20/$G$23</f>
-        <v>8.5552104701895626E-4</v>
-      </c>
-      <c r="I20" s="3"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
       <c r="J20" s="2"/>
-    </row>
-    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="6">
-        <v>65105</v>
-      </c>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="6">
-        <f>SUM(C21:F21)</f>
-        <v>65105</v>
-      </c>
-      <c r="H21" s="7">
-        <f>G21/$G$23</f>
-        <v>6.6841110963841528E-3</v>
-      </c>
-      <c r="I21" s="3"/>
+      <c r="B21" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="13">
+        <v>61746</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="E21" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-    </row>
-    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
+      <c r="B22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="13">
+        <v>100000</v>
+      </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
       <c r="J22" s="2"/>
-    </row>
-    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K22" s="2"/>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="13">
+        <v>100000</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="2"/>
+      <c r="B24" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="13">
+        <v>61746</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="2"/>
+      <c r="B25" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="13">
+        <v>250000</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="E25" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="2"/>
+      <c r="B27" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="9">
-        <f>SUM(C4:C21)</f>
-        <v>8629687</v>
-      </c>
-      <c r="D23" s="9">
-        <f>SUM(D4:D21)</f>
-        <v>879005</v>
-      </c>
-      <c r="E23" s="9">
-        <f>SUM(E4:E21)</f>
-        <v>210843</v>
-      </c>
-      <c r="F23" s="9">
-        <f>SUM(F4:F21)</f>
-        <v>20728</v>
-      </c>
-      <c r="G23" s="9">
-        <f>SUM(G4:G21)</f>
-        <v>9740263</v>
-      </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="2"/>
+      <c r="C27" s="12">
+        <f>SUM(C4:C25)</f>
+        <v>9825000</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>